<commit_message>
feat: selaraskan terminologi metrik ke 'ideal', perbarui visualisasi matriks D3 & Chart 15, dan rapikan rekapitulasi data
</commit_message>
<xml_diff>
--- a/data/processed/rekap_selisih_lulus_vs_daftar_ulang_2022_2026.xlsx
+++ b/data/processed/rekap_selisih_lulus_vs_daftar_ulang_2022_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan_Eksekutif" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rincian_Per_Prodi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ringkasan_Eksekutif" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Rincian_Per_Prodi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -176,8 +176,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="006D28D9"/>
+        <bgColor rgb="006D28D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B45309"/>
+        <bgColor rgb="00B45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0015803D"/>
+        <bgColor rgb="0015803D"/>
       </patternFill>
     </fill>
     <fill>
@@ -188,20 +200,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0015803D"/>
-        <bgColor rgb="0015803D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B45309"/>
-        <bgColor rgb="00B45309"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006D28D9"/>
-        <bgColor rgb="006D28D9"/>
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
     <fill>
@@ -212,8 +212,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002563EB"/>
-        <bgColor rgb="002563EB"/>
+        <fgColor rgb="007C3AED"/>
+        <bgColor rgb="007C3AED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D97706"/>
+        <bgColor rgb="00D97706"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0016A34A"/>
+        <bgColor rgb="0016A34A"/>
       </patternFill>
     </fill>
     <fill>
@@ -224,20 +236,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0016A34A"/>
-        <bgColor rgb="0016A34A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D97706"/>
-        <bgColor rgb="00D97706"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007C3AED"/>
-        <bgColor rgb="007C3AED"/>
+        <fgColor rgb="002563EB"/>
+        <bgColor rgb="002563EB"/>
       </patternFill>
     </fill>
     <fill>
@@ -1103,19 +1103,19 @@
         <v>2022</v>
       </c>
       <c r="B10" s="22">
-        <f>Rincian_Per_Prodi!E87</f>
+        <f>Rincian_Per_Prodi!U87</f>
         <v/>
       </c>
       <c r="C10" s="22">
-        <f>Rincian_Per_Prodi!F87</f>
+        <f>Rincian_Per_Prodi!V87</f>
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>Rincian_Per_Prodi!G87</f>
+        <f>Rincian_Per_Prodi!W87</f>
         <v/>
       </c>
       <c r="E10" s="23">
-        <f>Rincian_Per_Prodi!H87</f>
+        <f>Rincian_Per_Prodi!X87</f>
         <v/>
       </c>
       <c r="F10" s="23">
@@ -1132,19 +1132,19 @@
         <v>2023</v>
       </c>
       <c r="B11" s="25">
-        <f>Rincian_Per_Prodi!I87</f>
+        <f>Rincian_Per_Prodi!Q87</f>
         <v/>
       </c>
       <c r="C11" s="25">
-        <f>Rincian_Per_Prodi!J87</f>
+        <f>Rincian_Per_Prodi!R87</f>
         <v/>
       </c>
       <c r="D11" s="25">
-        <f>Rincian_Per_Prodi!K87</f>
+        <f>Rincian_Per_Prodi!S87</f>
         <v/>
       </c>
       <c r="E11" s="26">
-        <f>Rincian_Per_Prodi!L87</f>
+        <f>Rincian_Per_Prodi!T87</f>
         <v/>
       </c>
       <c r="F11" s="26">
@@ -1190,19 +1190,19 @@
         <v>2025</v>
       </c>
       <c r="B13" s="25">
-        <f>Rincian_Per_Prodi!Q87</f>
+        <f>Rincian_Per_Prodi!I87</f>
         <v/>
       </c>
       <c r="C13" s="25">
-        <f>Rincian_Per_Prodi!R87</f>
+        <f>Rincian_Per_Prodi!J87</f>
         <v/>
       </c>
       <c r="D13" s="25">
-        <f>Rincian_Per_Prodi!S87</f>
+        <f>Rincian_Per_Prodi!K87</f>
         <v/>
       </c>
       <c r="E13" s="26">
-        <f>Rincian_Per_Prodi!T87</f>
+        <f>Rincian_Per_Prodi!L87</f>
         <v/>
       </c>
       <c r="F13" s="26">
@@ -1219,19 +1219,19 @@
         <v>2026</v>
       </c>
       <c r="B14" s="22">
-        <f>Rincian_Per_Prodi!U87</f>
+        <f>Rincian_Per_Prodi!E87</f>
         <v/>
       </c>
       <c r="C14" s="22">
-        <f>Rincian_Per_Prodi!V87</f>
+        <f>Rincian_Per_Prodi!F87</f>
         <v/>
       </c>
       <c r="D14" s="22">
-        <f>Rincian_Per_Prodi!W87</f>
+        <f>Rincian_Per_Prodi!G87</f>
         <v/>
       </c>
       <c r="E14" s="23">
-        <f>Rincian_Per_Prodi!X87</f>
+        <f>Rincian_Per_Prodi!H87</f>
         <v/>
       </c>
       <c r="F14" s="23">
@@ -2305,7 +2305,7 @@
       <c r="D4" s="42" t="n"/>
       <c r="E4" s="43" t="inlineStr">
         <is>
-          <t>TAHUN AKADEMIK 2022</t>
+          <t>TAHUN AKADEMIK 2026</t>
         </is>
       </c>
       <c r="F4" s="44" t="n"/>
@@ -2313,7 +2313,7 @@
       <c r="H4" s="45" t="n"/>
       <c r="I4" s="46" t="inlineStr">
         <is>
-          <t>TAHUN AKADEMIK 2023</t>
+          <t>TAHUN AKADEMIK 2025</t>
         </is>
       </c>
       <c r="J4" s="47" t="n"/>
@@ -2329,7 +2329,7 @@
       <c r="P4" s="51" t="n"/>
       <c r="Q4" s="52" t="inlineStr">
         <is>
-          <t>TAHUN AKADEMIK 2025</t>
+          <t>TAHUN AKADEMIK 2023</t>
         </is>
       </c>
       <c r="R4" s="53" t="n"/>
@@ -2337,7 +2337,7 @@
       <c r="T4" s="54" t="n"/>
       <c r="U4" s="55" t="inlineStr">
         <is>
-          <t>TAHUN AKADEMIK 2026</t>
+          <t>TAHUN AKADEMIK 2022</t>
         </is>
       </c>
       <c r="V4" s="56" t="n"/>
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="E6" s="22" t="n">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>193</v>
+        <v>224</v>
       </c>
       <c r="G6" s="22">
         <f>MAX(0, E6-F6)</f>
@@ -2528,10 +2528,10 @@
         <v/>
       </c>
       <c r="I6" s="22" t="n">
-        <v>209</v>
+        <v>276</v>
       </c>
       <c r="J6" s="22" t="n">
-        <v>174</v>
+        <v>227</v>
       </c>
       <c r="K6" s="22">
         <f>MAX(0, I6-J6)</f>
@@ -2556,10 +2556,10 @@
         <v/>
       </c>
       <c r="Q6" s="22" t="n">
-        <v>276</v>
+        <v>209</v>
       </c>
       <c r="R6" s="22" t="n">
-        <v>227</v>
+        <v>174</v>
       </c>
       <c r="S6" s="22">
         <f>MAX(0, Q6-R6)</f>
@@ -2570,10 +2570,10 @@
         <v/>
       </c>
       <c r="U6" s="22" t="n">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="V6" s="22" t="n">
-        <v>224</v>
+        <v>193</v>
       </c>
       <c r="W6" s="22">
         <f>MAX(0, U6-V6)</f>
@@ -2620,10 +2620,10 @@
         </is>
       </c>
       <c r="E7" s="25" t="n">
-        <v>188</v>
+        <v>282</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>154</v>
+        <v>252</v>
       </c>
       <c r="G7" s="25">
         <f>MAX(0, E7-F7)</f>
@@ -2634,10 +2634,10 @@
         <v/>
       </c>
       <c r="I7" s="25" t="n">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="J7" s="25" t="n">
-        <v>169</v>
+        <v>232</v>
       </c>
       <c r="K7" s="25">
         <f>MAX(0, I7-J7)</f>
@@ -2662,10 +2662,10 @@
         <v/>
       </c>
       <c r="Q7" s="25" t="n">
-        <v>263</v>
+        <v>212</v>
       </c>
       <c r="R7" s="25" t="n">
-        <v>232</v>
+        <v>169</v>
       </c>
       <c r="S7" s="25">
         <f>MAX(0, Q7-R7)</f>
@@ -2676,10 +2676,10 @@
         <v/>
       </c>
       <c r="U7" s="25" t="n">
-        <v>282</v>
+        <v>188</v>
       </c>
       <c r="V7" s="25" t="n">
-        <v>252</v>
+        <v>154</v>
       </c>
       <c r="W7" s="25">
         <f>MAX(0, U7-V7)</f>
@@ -2729,7 +2729,7 @@
         <v>124</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G8" s="22">
         <f>MAX(0, E8-F8)</f>
@@ -2740,10 +2740,10 @@
         <v/>
       </c>
       <c r="I8" s="22" t="n">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="K8" s="22">
         <f>MAX(0, I8-J8)</f>
@@ -2768,10 +2768,10 @@
         <v/>
       </c>
       <c r="Q8" s="22" t="n">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="R8" s="22" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="S8" s="22">
         <f>MAX(0, Q8-R8)</f>
@@ -2785,7 +2785,7 @@
         <v>124</v>
       </c>
       <c r="V8" s="22" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="W8" s="22">
         <f>MAX(0, U8-V8)</f>
@@ -2832,10 +2832,10 @@
         </is>
       </c>
       <c r="E9" s="25" t="n">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="F9" s="25" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="G9" s="25">
         <f>MAX(0, E9-F9)</f>
@@ -2846,10 +2846,10 @@
         <v/>
       </c>
       <c r="I9" s="25" t="n">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="J9" s="25" t="n">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="K9" s="25">
         <f>MAX(0, I9-J9)</f>
@@ -2874,10 +2874,10 @@
         <v/>
       </c>
       <c r="Q9" s="25" t="n">
-        <v>143</v>
+        <v>108</v>
       </c>
       <c r="R9" s="25" t="n">
-        <v>116</v>
+        <v>85</v>
       </c>
       <c r="S9" s="25">
         <f>MAX(0, Q9-R9)</f>
@@ -2888,10 +2888,10 @@
         <v/>
       </c>
       <c r="U9" s="25" t="n">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="V9" s="25" t="n">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="W9" s="25">
         <f>MAX(0, U9-V9)</f>
@@ -2938,10 +2938,10 @@
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="G10" s="22">
         <f>MAX(0, E10-F10)</f>
@@ -2952,10 +2952,10 @@
         <v/>
       </c>
       <c r="I10" s="22" t="n">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="J10" s="22" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K10" s="22">
         <f>MAX(0, I10-J10)</f>
@@ -2980,10 +2980,10 @@
         <v/>
       </c>
       <c r="Q10" s="22" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="R10" s="22" t="n">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="S10" s="22">
         <f>MAX(0, Q10-R10)</f>
@@ -2994,10 +2994,10 @@
         <v/>
       </c>
       <c r="U10" s="22" t="n">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="V10" s="22" t="n">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="W10" s="22">
         <f>MAX(0, U10-V10)</f>
@@ -3044,10 +3044,10 @@
         </is>
       </c>
       <c r="E11" s="25" t="n">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="F11" s="25" t="n">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="G11" s="25">
         <f>MAX(0, E11-F11)</f>
@@ -3058,10 +3058,10 @@
         <v/>
       </c>
       <c r="I11" s="25" t="n">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="J11" s="25" t="n">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="K11" s="25">
         <f>MAX(0, I11-J11)</f>
@@ -3086,10 +3086,10 @@
         <v/>
       </c>
       <c r="Q11" s="25" t="n">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="R11" s="25" t="n">
-        <v>113</v>
+        <v>79</v>
       </c>
       <c r="S11" s="25">
         <f>MAX(0, Q11-R11)</f>
@@ -3100,10 +3100,10 @@
         <v/>
       </c>
       <c r="U11" s="25" t="n">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="V11" s="25" t="n">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="W11" s="25">
         <f>MAX(0, U11-V11)</f>
@@ -3150,10 +3150,10 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F12" s="22" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G12" s="22">
         <f>MAX(0, E12-F12)</f>
@@ -3164,10 +3164,10 @@
         <v/>
       </c>
       <c r="I12" s="22" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="J12" s="22" t="n">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="K12" s="22">
         <f>MAX(0, I12-J12)</f>
@@ -3192,10 +3192,10 @@
         <v/>
       </c>
       <c r="Q12" s="22" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="R12" s="22" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="S12" s="22">
         <f>MAX(0, Q12-R12)</f>
@@ -3206,10 +3206,10 @@
         <v/>
       </c>
       <c r="U12" s="22" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="V12" s="22" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="W12" s="22">
         <f>MAX(0, U12-V12)</f>
@@ -3256,10 +3256,10 @@
         </is>
       </c>
       <c r="E13" s="25" t="n">
-        <v>121</v>
+        <v>165</v>
       </c>
       <c r="F13" s="25" t="n">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="G13" s="25">
         <f>MAX(0, E13-F13)</f>
@@ -3270,10 +3270,10 @@
         <v/>
       </c>
       <c r="I13" s="25" t="n">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="K13" s="25">
         <f>MAX(0, I13-J13)</f>
@@ -3298,10 +3298,10 @@
         <v/>
       </c>
       <c r="Q13" s="25" t="n">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="R13" s="25" t="n">
-        <v>126</v>
+        <v>81</v>
       </c>
       <c r="S13" s="25">
         <f>MAX(0, Q13-R13)</f>
@@ -3312,10 +3312,10 @@
         <v/>
       </c>
       <c r="U13" s="25" t="n">
-        <v>165</v>
+        <v>121</v>
       </c>
       <c r="V13" s="25" t="n">
-        <v>135</v>
+        <v>98</v>
       </c>
       <c r="W13" s="25">
         <f>MAX(0, U13-V13)</f>
@@ -3362,10 +3362,10 @@
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="G14" s="22">
         <f>MAX(0, E14-F14)</f>
@@ -3376,10 +3376,10 @@
         <v/>
       </c>
       <c r="I14" s="22" t="n">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="J14" s="22" t="n">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="K14" s="22">
         <f>MAX(0, I14-J14)</f>
@@ -3404,10 +3404,10 @@
         <v/>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="R14" s="22" t="n">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="S14" s="22">
         <f>MAX(0, Q14-R14)</f>
@@ -3418,10 +3418,10 @@
         <v/>
       </c>
       <c r="U14" s="22" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="V14" s="22" t="n">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="W14" s="22">
         <f>MAX(0, U14-V14)</f>
@@ -3468,10 +3468,10 @@
         </is>
       </c>
       <c r="E15" s="25" t="n">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="F15" s="25" t="n">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G15" s="25">
         <f>MAX(0, E15-F15)</f>
@@ -3482,10 +3482,10 @@
         <v/>
       </c>
       <c r="I15" s="25" t="n">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="J15" s="25" t="n">
-        <v>60</v>
+        <v>102</v>
       </c>
       <c r="K15" s="25">
         <f>MAX(0, I15-J15)</f>
@@ -3510,10 +3510,10 @@
         <v/>
       </c>
       <c r="Q15" s="25" t="n">
-        <v>115</v>
+        <v>72</v>
       </c>
       <c r="R15" s="25" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="S15" s="25">
         <f>MAX(0, Q15-R15)</f>
@@ -3524,10 +3524,10 @@
         <v/>
       </c>
       <c r="U15" s="25" t="n">
-        <v>123</v>
+        <v>72</v>
       </c>
       <c r="V15" s="25" t="n">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="W15" s="25">
         <f>MAX(0, U15-V15)</f>
@@ -3574,10 +3574,10 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F16" s="22" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G16" s="22">
         <f>MAX(0, E16-F16)</f>
@@ -3588,10 +3588,10 @@
         <v/>
       </c>
       <c r="I16" s="22" t="n">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="J16" s="22" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="K16" s="22">
         <f>MAX(0, I16-J16)</f>
@@ -3616,10 +3616,10 @@
         <v/>
       </c>
       <c r="Q16" s="22" t="n">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="R16" s="22" t="n">
-        <v>118</v>
+        <v>85</v>
       </c>
       <c r="S16" s="22">
         <f>MAX(0, Q16-R16)</f>
@@ -3630,10 +3630,10 @@
         <v/>
       </c>
       <c r="U16" s="22" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="V16" s="22" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="W16" s="22">
         <f>MAX(0, U16-V16)</f>
@@ -3680,10 +3680,10 @@
         </is>
       </c>
       <c r="E17" s="25" t="n">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="F17" s="25" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G17" s="25">
         <f>MAX(0, E17-F17)</f>
@@ -3694,7 +3694,7 @@
         <v/>
       </c>
       <c r="I17" s="25" t="n">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="J17" s="25" t="n">
         <v>82</v>
@@ -3722,7 +3722,7 @@
         <v/>
       </c>
       <c r="Q17" s="25" t="n">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="R17" s="25" t="n">
         <v>82</v>
@@ -3736,10 +3736,10 @@
         <v/>
       </c>
       <c r="U17" s="25" t="n">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="V17" s="25" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="W17" s="25">
         <f>MAX(0, U17-V17)</f>
@@ -3786,10 +3786,10 @@
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="F18" s="22" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G18" s="22">
         <f>MAX(0, E18-F18)</f>
@@ -3800,10 +3800,10 @@
         <v/>
       </c>
       <c r="I18" s="22" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="J18" s="22" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="K18" s="22">
         <f>MAX(0, I18-J18)</f>
@@ -3828,10 +3828,10 @@
         <v/>
       </c>
       <c r="Q18" s="22" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="R18" s="22" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="S18" s="22">
         <f>MAX(0, Q18-R18)</f>
@@ -3842,10 +3842,10 @@
         <v/>
       </c>
       <c r="U18" s="22" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="V18" s="22" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="W18" s="22">
         <f>MAX(0, U18-V18)</f>
@@ -3892,10 +3892,10 @@
         </is>
       </c>
       <c r="E19" s="25" t="n">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="G19" s="25">
         <f>MAX(0, E19-F19)</f>
@@ -3906,10 +3906,10 @@
         <v/>
       </c>
       <c r="I19" s="25" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="J19" s="25" t="n">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="K19" s="25">
         <f>MAX(0, I19-J19)</f>
@@ -3934,10 +3934,10 @@
         <v/>
       </c>
       <c r="Q19" s="25" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="R19" s="25" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="S19" s="25">
         <f>MAX(0, Q19-R19)</f>
@@ -3948,10 +3948,10 @@
         <v/>
       </c>
       <c r="U19" s="25" t="n">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="V19" s="25" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="W19" s="25">
         <f>MAX(0, U19-V19)</f>
@@ -3998,10 +3998,10 @@
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F20" s="22" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="G20" s="22">
         <f>MAX(0, E20-F20)</f>
@@ -4012,10 +4012,10 @@
         <v/>
       </c>
       <c r="I20" s="22" t="n">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="J20" s="22" t="n">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="K20" s="22">
         <f>MAX(0, I20-J20)</f>
@@ -4040,10 +4040,10 @@
         <v/>
       </c>
       <c r="Q20" s="22" t="n">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="R20" s="22" t="n">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="S20" s="22">
         <f>MAX(0, Q20-R20)</f>
@@ -4054,10 +4054,10 @@
         <v/>
       </c>
       <c r="U20" s="22" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="V20" s="22" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="W20" s="22">
         <f>MAX(0, U20-V20)</f>
@@ -4104,10 +4104,10 @@
         </is>
       </c>
       <c r="E21" s="25" t="n">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="F21" s="25" t="n">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="G21" s="25">
         <f>MAX(0, E21-F21)</f>
@@ -4118,10 +4118,10 @@
         <v/>
       </c>
       <c r="I21" s="25" t="n">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="J21" s="25" t="n">
-        <v>213</v>
+        <v>254</v>
       </c>
       <c r="K21" s="25">
         <f>MAX(0, I21-J21)</f>
@@ -4146,10 +4146,10 @@
         <v/>
       </c>
       <c r="Q21" s="25" t="n">
-        <v>278</v>
+        <v>253</v>
       </c>
       <c r="R21" s="25" t="n">
-        <v>254</v>
+        <v>213</v>
       </c>
       <c r="S21" s="25">
         <f>MAX(0, Q21-R21)</f>
@@ -4160,10 +4160,10 @@
         <v/>
       </c>
       <c r="U21" s="25" t="n">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="V21" s="25" t="n">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="W21" s="25">
         <f>MAX(0, U21-V21)</f>
@@ -4210,10 +4210,10 @@
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>167</v>
+        <v>373</v>
       </c>
       <c r="F22" s="22" t="n">
-        <v>127</v>
+        <v>295</v>
       </c>
       <c r="G22" s="22">
         <f>MAX(0, E22-F22)</f>
@@ -4224,10 +4224,10 @@
         <v/>
       </c>
       <c r="I22" s="22" t="n">
-        <v>207</v>
+        <v>371</v>
       </c>
       <c r="J22" s="22" t="n">
-        <v>164</v>
+        <v>280</v>
       </c>
       <c r="K22" s="22">
         <f>MAX(0, I22-J22)</f>
@@ -4252,10 +4252,10 @@
         <v/>
       </c>
       <c r="Q22" s="22" t="n">
-        <v>371</v>
+        <v>207</v>
       </c>
       <c r="R22" s="22" t="n">
-        <v>280</v>
+        <v>164</v>
       </c>
       <c r="S22" s="22">
         <f>MAX(0, Q22-R22)</f>
@@ -4266,10 +4266,10 @@
         <v/>
       </c>
       <c r="U22" s="22" t="n">
-        <v>373</v>
+        <v>167</v>
       </c>
       <c r="V22" s="22" t="n">
-        <v>295</v>
+        <v>127</v>
       </c>
       <c r="W22" s="22">
         <f>MAX(0, U22-V22)</f>
@@ -4316,10 +4316,10 @@
         </is>
       </c>
       <c r="E23" s="25" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="G23" s="25">
         <f>MAX(0, E23-F23)</f>
@@ -4330,10 +4330,10 @@
         <v/>
       </c>
       <c r="I23" s="25" t="n">
+        <v>108</v>
+      </c>
+      <c r="J23" s="25" t="n">
         <v>101</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>83</v>
       </c>
       <c r="K23" s="25">
         <f>MAX(0, I23-J23)</f>
@@ -4358,10 +4358,10 @@
         <v/>
       </c>
       <c r="Q23" s="25" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="R23" s="25" t="n">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="S23" s="25">
         <f>MAX(0, Q23-R23)</f>
@@ -4372,10 +4372,10 @@
         <v/>
       </c>
       <c r="U23" s="25" t="n">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="V23" s="25" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="W23" s="25">
         <f>MAX(0, U23-V23)</f>
@@ -4422,10 +4422,10 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="F24" s="22" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G24" s="22">
         <f>MAX(0, E24-F24)</f>
@@ -4436,10 +4436,10 @@
         <v/>
       </c>
       <c r="I24" s="22" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="J24" s="22" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K24" s="22">
         <f>MAX(0, I24-J24)</f>
@@ -4464,10 +4464,10 @@
         <v/>
       </c>
       <c r="Q24" s="22" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="R24" s="22" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="S24" s="22">
         <f>MAX(0, Q24-R24)</f>
@@ -4478,10 +4478,10 @@
         <v/>
       </c>
       <c r="U24" s="22" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="V24" s="22" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="W24" s="22">
         <f>MAX(0, U24-V24)</f>
@@ -4528,7 +4528,7 @@
         </is>
       </c>
       <c r="E25" s="25" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F25" s="25" t="n">
         <v>42</v>
@@ -4542,10 +4542,10 @@
         <v/>
       </c>
       <c r="I25" s="25" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="J25" s="25" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="K25" s="25">
         <f>MAX(0, I25-J25)</f>
@@ -4570,10 +4570,10 @@
         <v/>
       </c>
       <c r="Q25" s="25" t="n">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="R25" s="25" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="S25" s="25">
         <f>MAX(0, Q25-R25)</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="U25" s="25" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="V25" s="25" t="n">
         <v>42</v>
@@ -4634,10 +4634,10 @@
         </is>
       </c>
       <c r="E26" s="22" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F26" s="22" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G26" s="22">
         <f>MAX(0, E26-F26)</f>
@@ -4648,10 +4648,10 @@
         <v/>
       </c>
       <c r="I26" s="22" t="n">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="J26" s="22" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="K26" s="22">
         <f>MAX(0, I26-J26)</f>
@@ -4676,10 +4676,10 @@
         <v/>
       </c>
       <c r="Q26" s="22" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="R26" s="22" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="S26" s="22">
         <f>MAX(0, Q26-R26)</f>
@@ -4690,10 +4690,10 @@
         <v/>
       </c>
       <c r="U26" s="22" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="V26" s="22" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="W26" s="22">
         <f>MAX(0, U26-V26)</f>
@@ -4740,10 +4740,10 @@
         </is>
       </c>
       <c r="E27" s="25" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F27" s="25" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G27" s="25">
         <f>MAX(0, E27-F27)</f>
@@ -4754,10 +4754,10 @@
         <v/>
       </c>
       <c r="I27" s="25" t="n">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="J27" s="25" t="n">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="K27" s="25">
         <f>MAX(0, I27-J27)</f>
@@ -4782,10 +4782,10 @@
         <v/>
       </c>
       <c r="Q27" s="25" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="R27" s="25" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="S27" s="25">
         <f>MAX(0, Q27-R27)</f>
@@ -4796,10 +4796,10 @@
         <v/>
       </c>
       <c r="U27" s="25" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="V27" s="25" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="W27" s="25">
         <f>MAX(0, U27-V27)</f>
@@ -4846,10 +4846,10 @@
         </is>
       </c>
       <c r="E28" s="22" t="n">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="F28" s="22" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="G28" s="22">
         <f>MAX(0, E28-F28)</f>
@@ -4860,10 +4860,10 @@
         <v/>
       </c>
       <c r="I28" s="22" t="n">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="J28" s="22" t="n">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="K28" s="22">
         <f>MAX(0, I28-J28)</f>
@@ -4888,10 +4888,10 @@
         <v/>
       </c>
       <c r="Q28" s="22" t="n">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="R28" s="22" t="n">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="S28" s="22">
         <f>MAX(0, Q28-R28)</f>
@@ -4902,10 +4902,10 @@
         <v/>
       </c>
       <c r="U28" s="22" t="n">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="V28" s="22" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="W28" s="22">
         <f>MAX(0, U28-V28)</f>
@@ -4952,7 +4952,7 @@
         </is>
       </c>
       <c r="E29" s="25" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F29" s="25" t="n">
         <v>90</v>
@@ -4966,10 +4966,10 @@
         <v/>
       </c>
       <c r="I29" s="25" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="K29" s="25">
         <f>MAX(0, I29-J29)</f>
@@ -4994,10 +4994,10 @@
         <v/>
       </c>
       <c r="Q29" s="25" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="R29" s="25" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="S29" s="25">
         <f>MAX(0, Q29-R29)</f>
@@ -5008,7 +5008,7 @@
         <v/>
       </c>
       <c r="U29" s="25" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="V29" s="25" t="n">
         <v>90</v>
@@ -5058,10 +5058,10 @@
         </is>
       </c>
       <c r="E30" s="22" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="F30" s="22" t="n">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="G30" s="22">
         <f>MAX(0, E30-F30)</f>
@@ -5072,10 +5072,10 @@
         <v/>
       </c>
       <c r="I30" s="22" t="n">
-        <v>88</v>
+        <v>131</v>
       </c>
       <c r="J30" s="22" t="n">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="K30" s="22">
         <f>MAX(0, I30-J30)</f>
@@ -5100,10 +5100,10 @@
         <v/>
       </c>
       <c r="Q30" s="22" t="n">
-        <v>131</v>
+        <v>88</v>
       </c>
       <c r="R30" s="22" t="n">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="S30" s="22">
         <f>MAX(0, Q30-R30)</f>
@@ -5114,10 +5114,10 @@
         <v/>
       </c>
       <c r="U30" s="22" t="n">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="V30" s="22" t="n">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="W30" s="22">
         <f>MAX(0, U30-V30)</f>
@@ -5164,10 +5164,10 @@
         </is>
       </c>
       <c r="E31" s="25" t="n">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="F31" s="25" t="n">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="G31" s="25">
         <f>MAX(0, E31-F31)</f>
@@ -5178,10 +5178,10 @@
         <v/>
       </c>
       <c r="I31" s="25" t="n">
-        <v>91</v>
+        <v>135</v>
       </c>
       <c r="J31" s="25" t="n">
-        <v>78</v>
+        <v>116</v>
       </c>
       <c r="K31" s="25">
         <f>MAX(0, I31-J31)</f>
@@ -5206,10 +5206,10 @@
         <v/>
       </c>
       <c r="Q31" s="25" t="n">
-        <v>135</v>
+        <v>91</v>
       </c>
       <c r="R31" s="25" t="n">
-        <v>116</v>
+        <v>78</v>
       </c>
       <c r="S31" s="25">
         <f>MAX(0, Q31-R31)</f>
@@ -5220,10 +5220,10 @@
         <v/>
       </c>
       <c r="U31" s="25" t="n">
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="V31" s="25" t="n">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="W31" s="25">
         <f>MAX(0, U31-V31)</f>
@@ -5270,10 +5270,10 @@
         </is>
       </c>
       <c r="E32" s="22" t="n">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="F32" s="22" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="G32" s="22">
         <f>MAX(0, E32-F32)</f>
@@ -5284,10 +5284,10 @@
         <v/>
       </c>
       <c r="I32" s="22" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="J32" s="22" t="n">
-        <v>52</v>
+        <v>82</v>
       </c>
       <c r="K32" s="22">
         <f>MAX(0, I32-J32)</f>
@@ -5312,10 +5312,10 @@
         <v/>
       </c>
       <c r="Q32" s="22" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="R32" s="22" t="n">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="S32" s="22">
         <f>MAX(0, Q32-R32)</f>
@@ -5326,10 +5326,10 @@
         <v/>
       </c>
       <c r="U32" s="22" t="n">
-        <v>102</v>
+        <v>72</v>
       </c>
       <c r="V32" s="22" t="n">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="W32" s="22">
         <f>MAX(0, U32-V32)</f>
@@ -5376,10 +5376,10 @@
         </is>
       </c>
       <c r="E33" s="25" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="F33" s="25" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="G33" s="25">
         <f>MAX(0, E33-F33)</f>
@@ -5390,10 +5390,10 @@
         <v/>
       </c>
       <c r="I33" s="25" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J33" s="25" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="K33" s="25">
         <f>MAX(0, I33-J33)</f>
@@ -5418,10 +5418,10 @@
         <v/>
       </c>
       <c r="Q33" s="25" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="R33" s="25" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="S33" s="25">
         <f>MAX(0, Q33-R33)</f>
@@ -5432,10 +5432,10 @@
         <v/>
       </c>
       <c r="U33" s="25" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="V33" s="25" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="W33" s="25">
         <f>MAX(0, U33-V33)</f>
@@ -5482,10 +5482,10 @@
         </is>
       </c>
       <c r="E34" s="22" t="n">
-        <v>85</v>
+        <v>138</v>
       </c>
       <c r="F34" s="22" t="n">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="G34" s="22">
         <f>MAX(0, E34-F34)</f>
@@ -5496,10 +5496,10 @@
         <v/>
       </c>
       <c r="I34" s="22" t="n">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="J34" s="22" t="n">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K34" s="22">
         <f>MAX(0, I34-J34)</f>
@@ -5524,10 +5524,10 @@
         <v/>
       </c>
       <c r="Q34" s="22" t="n">
-        <v>130</v>
+        <v>91</v>
       </c>
       <c r="R34" s="22" t="n">
-        <v>113</v>
+        <v>75</v>
       </c>
       <c r="S34" s="22">
         <f>MAX(0, Q34-R34)</f>
@@ -5538,10 +5538,10 @@
         <v/>
       </c>
       <c r="U34" s="22" t="n">
-        <v>138</v>
+        <v>85</v>
       </c>
       <c r="V34" s="22" t="n">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="W34" s="22">
         <f>MAX(0, U34-V34)</f>
@@ -5588,10 +5588,10 @@
         </is>
       </c>
       <c r="E35" s="25" t="n">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="F35" s="25" t="n">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="G35" s="25">
         <f>MAX(0, E35-F35)</f>
@@ -5602,10 +5602,10 @@
         <v/>
       </c>
       <c r="I35" s="25" t="n">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="J35" s="25" t="n">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="K35" s="25">
         <f>MAX(0, I35-J35)</f>
@@ -5630,10 +5630,10 @@
         <v/>
       </c>
       <c r="Q35" s="25" t="n">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="R35" s="25" t="n">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="S35" s="25">
         <f>MAX(0, Q35-R35)</f>
@@ -5644,10 +5644,10 @@
         <v/>
       </c>
       <c r="U35" s="25" t="n">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="V35" s="25" t="n">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="W35" s="25">
         <f>MAX(0, U35-V35)</f>
@@ -5694,10 +5694,10 @@
         </is>
       </c>
       <c r="E36" s="22" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F36" s="22" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="G36" s="22">
         <f>MAX(0, E36-F36)</f>
@@ -5708,10 +5708,10 @@
         <v/>
       </c>
       <c r="I36" s="22" t="n">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="J36" s="22" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="K36" s="22">
         <f>MAX(0, I36-J36)</f>
@@ -5736,10 +5736,10 @@
         <v/>
       </c>
       <c r="Q36" s="22" t="n">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="R36" s="22" t="n">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="S36" s="22">
         <f>MAX(0, Q36-R36)</f>
@@ -5750,10 +5750,10 @@
         <v/>
       </c>
       <c r="U36" s="22" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="V36" s="22" t="n">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="W36" s="22">
         <f>MAX(0, U36-V36)</f>
@@ -5800,10 +5800,10 @@
         </is>
       </c>
       <c r="E37" s="25" t="n">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="F37" s="25" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="G37" s="25">
         <f>MAX(0, E37-F37)</f>
@@ -5814,10 +5814,10 @@
         <v/>
       </c>
       <c r="I37" s="25" t="n">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="K37" s="25">
         <f>MAX(0, I37-J37)</f>
@@ -5842,10 +5842,10 @@
         <v/>
       </c>
       <c r="Q37" s="25" t="n">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="R37" s="25" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="S37" s="25">
         <f>MAX(0, Q37-R37)</f>
@@ -5856,10 +5856,10 @@
         <v/>
       </c>
       <c r="U37" s="25" t="n">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="V37" s="25" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="W37" s="25">
         <f>MAX(0, U37-V37)</f>
@@ -5906,10 +5906,10 @@
         </is>
       </c>
       <c r="E38" s="22" t="n">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="F38" s="22" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="G38" s="22">
         <f>MAX(0, E38-F38)</f>
@@ -5920,10 +5920,10 @@
         <v/>
       </c>
       <c r="I38" s="22" t="n">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="J38" s="22" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="K38" s="22">
         <f>MAX(0, I38-J38)</f>
@@ -5948,10 +5948,10 @@
         <v/>
       </c>
       <c r="Q38" s="22" t="n">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="R38" s="22" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="S38" s="22">
         <f>MAX(0, Q38-R38)</f>
@@ -5962,10 +5962,10 @@
         <v/>
       </c>
       <c r="U38" s="22" t="n">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="V38" s="22" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="W38" s="22">
         <f>MAX(0, U38-V38)</f>
@@ -6012,10 +6012,10 @@
         </is>
       </c>
       <c r="E39" s="25" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F39" s="25" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G39" s="25">
         <f>MAX(0, E39-F39)</f>
@@ -6026,10 +6026,10 @@
         <v/>
       </c>
       <c r="I39" s="25" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="J39" s="25" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K39" s="25">
         <f>MAX(0, I39-J39)</f>
@@ -6054,10 +6054,10 @@
         <v/>
       </c>
       <c r="Q39" s="25" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="R39" s="25" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="S39" s="25">
         <f>MAX(0, Q39-R39)</f>
@@ -6068,10 +6068,10 @@
         <v/>
       </c>
       <c r="U39" s="25" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="V39" s="25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="W39" s="25">
         <f>MAX(0, U39-V39)</f>
@@ -6118,10 +6118,10 @@
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F40" s="22" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="G40" s="22">
         <f>MAX(0, E40-F40)</f>
@@ -6132,10 +6132,10 @@
         <v/>
       </c>
       <c r="I40" s="22" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J40" s="22" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K40" s="22">
         <f>MAX(0, I40-J40)</f>
@@ -6160,10 +6160,10 @@
         <v/>
       </c>
       <c r="Q40" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="R40" s="22" t="n">
         <v>13</v>
-      </c>
-      <c r="R40" s="22" t="n">
-        <v>11</v>
       </c>
       <c r="S40" s="22">
         <f>MAX(0, Q40-R40)</f>
@@ -6174,10 +6174,10 @@
         <v/>
       </c>
       <c r="U40" s="22" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="V40" s="22" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="W40" s="22">
         <f>MAX(0, U40-V40)</f>
@@ -6224,10 +6224,10 @@
         </is>
       </c>
       <c r="E41" s="25" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F41" s="25" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G41" s="25">
         <f>MAX(0, E41-F41)</f>
@@ -6238,10 +6238,10 @@
         <v/>
       </c>
       <c r="I41" s="25" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="J41" s="25" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="K41" s="25">
         <f>MAX(0, I41-J41)</f>
@@ -6266,10 +6266,10 @@
         <v/>
       </c>
       <c r="Q41" s="25" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="R41" s="25" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="S41" s="25">
         <f>MAX(0, Q41-R41)</f>
@@ -6280,10 +6280,10 @@
         <v/>
       </c>
       <c r="U41" s="25" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="V41" s="25" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="W41" s="25">
         <f>MAX(0, U41-V41)</f>
@@ -6330,10 +6330,10 @@
         </is>
       </c>
       <c r="E42" s="22" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F42" s="22" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G42" s="22">
         <f>MAX(0, E42-F42)</f>
@@ -6344,10 +6344,10 @@
         <v/>
       </c>
       <c r="I42" s="22" t="n">
+        <v>58</v>
+      </c>
+      <c r="J42" s="22" t="n">
         <v>48</v>
-      </c>
-      <c r="J42" s="22" t="n">
-        <v>37</v>
       </c>
       <c r="K42" s="22">
         <f>MAX(0, I42-J42)</f>
@@ -6372,10 +6372,10 @@
         <v/>
       </c>
       <c r="Q42" s="22" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="R42" s="22" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="S42" s="22">
         <f>MAX(0, Q42-R42)</f>
@@ -6386,10 +6386,10 @@
         <v/>
       </c>
       <c r="U42" s="22" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="V42" s="22" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="W42" s="22">
         <f>MAX(0, U42-V42)</f>
@@ -6436,10 +6436,10 @@
         </is>
       </c>
       <c r="E43" s="25" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="F43" s="25" t="n">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="G43" s="25">
         <f>MAX(0, E43-F43)</f>
@@ -6450,10 +6450,10 @@
         <v/>
       </c>
       <c r="I43" s="25" t="n">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="J43" s="25" t="n">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="K43" s="25">
         <f>MAX(0, I43-J43)</f>
@@ -6478,10 +6478,10 @@
         <v/>
       </c>
       <c r="Q43" s="25" t="n">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="R43" s="25" t="n">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="S43" s="25">
         <f>MAX(0, Q43-R43)</f>
@@ -6492,10 +6492,10 @@
         <v/>
       </c>
       <c r="U43" s="25" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="V43" s="25" t="n">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="W43" s="25">
         <f>MAX(0, U43-V43)</f>
@@ -6542,10 +6542,10 @@
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="F44" s="22" t="n">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="G44" s="22">
         <f>MAX(0, E44-F44)</f>
@@ -6556,10 +6556,10 @@
         <v/>
       </c>
       <c r="I44" s="22" t="n">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="J44" s="22" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="K44" s="22">
         <f>MAX(0, I44-J44)</f>
@@ -6584,10 +6584,10 @@
         <v/>
       </c>
       <c r="Q44" s="22" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="R44" s="22" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="S44" s="22">
         <f>MAX(0, Q44-R44)</f>
@@ -6598,10 +6598,10 @@
         <v/>
       </c>
       <c r="U44" s="22" t="n">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="V44" s="22" t="n">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="W44" s="22">
         <f>MAX(0, U44-V44)</f>
@@ -6648,10 +6648,10 @@
         </is>
       </c>
       <c r="E45" s="25" t="n">
-        <v>110</v>
+        <v>186</v>
       </c>
       <c r="F45" s="25" t="n">
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="G45" s="25">
         <f>MAX(0, E45-F45)</f>
@@ -6662,10 +6662,10 @@
         <v/>
       </c>
       <c r="I45" s="25" t="n">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="J45" s="25" t="n">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="K45" s="25">
         <f>MAX(0, I45-J45)</f>
@@ -6690,10 +6690,10 @@
         <v/>
       </c>
       <c r="Q45" s="25" t="n">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="R45" s="25" t="n">
-        <v>136</v>
+        <v>100</v>
       </c>
       <c r="S45" s="25">
         <f>MAX(0, Q45-R45)</f>
@@ -6704,10 +6704,10 @@
         <v/>
       </c>
       <c r="U45" s="25" t="n">
-        <v>186</v>
+        <v>110</v>
       </c>
       <c r="V45" s="25" t="n">
-        <v>145</v>
+        <v>85</v>
       </c>
       <c r="W45" s="25">
         <f>MAX(0, U45-V45)</f>
@@ -6754,10 +6754,10 @@
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>202</v>
+        <v>151</v>
       </c>
       <c r="F46" s="22" t="n">
-        <v>169</v>
+        <v>135</v>
       </c>
       <c r="G46" s="22">
         <f>MAX(0, E46-F46)</f>
@@ -6768,10 +6768,10 @@
         <v/>
       </c>
       <c r="I46" s="22" t="n">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="J46" s="22" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="K46" s="22">
         <f>MAX(0, I46-J46)</f>
@@ -6796,10 +6796,10 @@
         <v/>
       </c>
       <c r="Q46" s="22" t="n">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="R46" s="22" t="n">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="S46" s="22">
         <f>MAX(0, Q46-R46)</f>
@@ -6810,10 +6810,10 @@
         <v/>
       </c>
       <c r="U46" s="22" t="n">
-        <v>151</v>
+        <v>202</v>
       </c>
       <c r="V46" s="22" t="n">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="W46" s="22">
         <f>MAX(0, U46-V46)</f>
@@ -6860,10 +6860,10 @@
         </is>
       </c>
       <c r="E47" s="25" t="n">
-        <v>298</v>
+        <v>226</v>
       </c>
       <c r="F47" s="25" t="n">
-        <v>266</v>
+        <v>199</v>
       </c>
       <c r="G47" s="25">
         <f>MAX(0, E47-F47)</f>
@@ -6874,10 +6874,10 @@
         <v/>
       </c>
       <c r="I47" s="25" t="n">
-        <v>275</v>
+        <v>214</v>
       </c>
       <c r="J47" s="25" t="n">
-        <v>227</v>
+        <v>199</v>
       </c>
       <c r="K47" s="25">
         <f>MAX(0, I47-J47)</f>
@@ -6902,10 +6902,10 @@
         <v/>
       </c>
       <c r="Q47" s="25" t="n">
-        <v>214</v>
+        <v>275</v>
       </c>
       <c r="R47" s="25" t="n">
-        <v>199</v>
+        <v>227</v>
       </c>
       <c r="S47" s="25">
         <f>MAX(0, Q47-R47)</f>
@@ -6916,10 +6916,10 @@
         <v/>
       </c>
       <c r="U47" s="25" t="n">
-        <v>226</v>
+        <v>298</v>
       </c>
       <c r="V47" s="25" t="n">
-        <v>199</v>
+        <v>266</v>
       </c>
       <c r="W47" s="25">
         <f>MAX(0, U47-V47)</f>
@@ -6966,10 +6966,10 @@
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F48" s="22" t="n">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="G48" s="22">
         <f>MAX(0, E48-F48)</f>
@@ -6980,10 +6980,10 @@
         <v/>
       </c>
       <c r="I48" s="22" t="n">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="J48" s="22" t="n">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="K48" s="22">
         <f>MAX(0, I48-J48)</f>
@@ -7008,10 +7008,10 @@
         <v/>
       </c>
       <c r="Q48" s="22" t="n">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="R48" s="22" t="n">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="S48" s="22">
         <f>MAX(0, Q48-R48)</f>
@@ -7022,10 +7022,10 @@
         <v/>
       </c>
       <c r="U48" s="22" t="n">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="V48" s="22" t="n">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="W48" s="22">
         <f>MAX(0, U48-V48)</f>
@@ -7072,10 +7072,10 @@
         </is>
       </c>
       <c r="E49" s="25" t="n">
-        <v>452</v>
+        <v>613</v>
       </c>
       <c r="F49" s="25" t="n">
-        <v>423</v>
+        <v>558</v>
       </c>
       <c r="G49" s="25">
         <f>MAX(0, E49-F49)</f>
@@ -7086,10 +7086,10 @@
         <v/>
       </c>
       <c r="I49" s="25" t="n">
-        <v>513</v>
+        <v>608</v>
       </c>
       <c r="J49" s="25" t="n">
-        <v>459</v>
+        <v>552</v>
       </c>
       <c r="K49" s="25">
         <f>MAX(0, I49-J49)</f>
@@ -7114,10 +7114,10 @@
         <v/>
       </c>
       <c r="Q49" s="25" t="n">
-        <v>608</v>
+        <v>513</v>
       </c>
       <c r="R49" s="25" t="n">
-        <v>552</v>
+        <v>459</v>
       </c>
       <c r="S49" s="25">
         <f>MAX(0, Q49-R49)</f>
@@ -7128,10 +7128,10 @@
         <v/>
       </c>
       <c r="U49" s="25" t="n">
-        <v>613</v>
+        <v>452</v>
       </c>
       <c r="V49" s="25" t="n">
-        <v>558</v>
+        <v>423</v>
       </c>
       <c r="W49" s="25">
         <f>MAX(0, U49-V49)</f>
@@ -7178,10 +7178,10 @@
         </is>
       </c>
       <c r="E50" s="22" t="n">
-        <v>92</v>
+        <v>143</v>
       </c>
       <c r="F50" s="22" t="n">
-        <v>77</v>
+        <v>129</v>
       </c>
       <c r="G50" s="22">
         <f>MAX(0, E50-F50)</f>
@@ -7192,10 +7192,10 @@
         <v/>
       </c>
       <c r="I50" s="22" t="n">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="J50" s="22" t="n">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="K50" s="22">
         <f>MAX(0, I50-J50)</f>
@@ -7220,10 +7220,10 @@
         <v/>
       </c>
       <c r="Q50" s="22" t="n">
-        <v>126</v>
+        <v>94</v>
       </c>
       <c r="R50" s="22" t="n">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="S50" s="22">
         <f>MAX(0, Q50-R50)</f>
@@ -7234,10 +7234,10 @@
         <v/>
       </c>
       <c r="U50" s="22" t="n">
-        <v>143</v>
+        <v>92</v>
       </c>
       <c r="V50" s="22" t="n">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="W50" s="22">
         <f>MAX(0, U50-V50)</f>
@@ -7284,10 +7284,10 @@
         </is>
       </c>
       <c r="E51" s="25" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F51" s="25" t="n">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G51" s="25">
         <f>MAX(0, E51-F51)</f>
@@ -7298,10 +7298,10 @@
         <v/>
       </c>
       <c r="I51" s="25" t="n">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="J51" s="25" t="n">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="K51" s="25">
         <f>MAX(0, I51-J51)</f>
@@ -7326,10 +7326,10 @@
         <v/>
       </c>
       <c r="Q51" s="25" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="R51" s="25" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="S51" s="25">
         <f>MAX(0, Q51-R51)</f>
@@ -7340,10 +7340,10 @@
         <v/>
       </c>
       <c r="U51" s="25" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="V51" s="25" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="W51" s="25">
         <f>MAX(0, U51-V51)</f>
@@ -7390,10 +7390,10 @@
         </is>
       </c>
       <c r="E52" s="22" t="n">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="F52" s="22" t="n">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="G52" s="22">
         <f>MAX(0, E52-F52)</f>
@@ -7404,10 +7404,10 @@
         <v/>
       </c>
       <c r="I52" s="22" t="n">
-        <v>93</v>
+        <v>128</v>
       </c>
       <c r="J52" s="22" t="n">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="K52" s="22">
         <f>MAX(0, I52-J52)</f>
@@ -7432,10 +7432,10 @@
         <v/>
       </c>
       <c r="Q52" s="22" t="n">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="R52" s="22" t="n">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="S52" s="22">
         <f>MAX(0, Q52-R52)</f>
@@ -7446,10 +7446,10 @@
         <v/>
       </c>
       <c r="U52" s="22" t="n">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="V52" s="22" t="n">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="W52" s="22">
         <f>MAX(0, U52-V52)</f>
@@ -7496,10 +7496,10 @@
         </is>
       </c>
       <c r="E53" s="25" t="n">
-        <v>82</v>
+        <v>129</v>
       </c>
       <c r="F53" s="25" t="n">
-        <v>71</v>
+        <v>119</v>
       </c>
       <c r="G53" s="25">
         <f>MAX(0, E53-F53)</f>
@@ -7510,10 +7510,10 @@
         <v/>
       </c>
       <c r="I53" s="25" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="J53" s="25" t="n">
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="K53" s="25">
         <f>MAX(0, I53-J53)</f>
@@ -7538,10 +7538,10 @@
         <v/>
       </c>
       <c r="Q53" s="25" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="R53" s="25" t="n">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="S53" s="25">
         <f>MAX(0, Q53-R53)</f>
@@ -7552,10 +7552,10 @@
         <v/>
       </c>
       <c r="U53" s="25" t="n">
-        <v>129</v>
+        <v>82</v>
       </c>
       <c r="V53" s="25" t="n">
-        <v>119</v>
+        <v>71</v>
       </c>
       <c r="W53" s="25">
         <f>MAX(0, U53-V53)</f>
@@ -7602,10 +7602,10 @@
         </is>
       </c>
       <c r="E54" s="22" t="n">
-        <v>85</v>
+        <v>154</v>
       </c>
       <c r="F54" s="22" t="n">
-        <v>64</v>
+        <v>134</v>
       </c>
       <c r="G54" s="22">
         <f>MAX(0, E54-F54)</f>
@@ -7616,10 +7616,10 @@
         <v/>
       </c>
       <c r="I54" s="22" t="n">
-        <v>94</v>
+        <v>137</v>
       </c>
       <c r="J54" s="22" t="n">
-        <v>82</v>
+        <v>124</v>
       </c>
       <c r="K54" s="22">
         <f>MAX(0, I54-J54)</f>
@@ -7644,10 +7644,10 @@
         <v/>
       </c>
       <c r="Q54" s="22" t="n">
-        <v>137</v>
+        <v>94</v>
       </c>
       <c r="R54" s="22" t="n">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="S54" s="22">
         <f>MAX(0, Q54-R54)</f>
@@ -7658,10 +7658,10 @@
         <v/>
       </c>
       <c r="U54" s="22" t="n">
-        <v>154</v>
+        <v>85</v>
       </c>
       <c r="V54" s="22" t="n">
-        <v>134</v>
+        <v>64</v>
       </c>
       <c r="W54" s="22">
         <f>MAX(0, U54-V54)</f>
@@ -7708,10 +7708,10 @@
         </is>
       </c>
       <c r="E55" s="25" t="n">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="F55" s="25" t="n">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="G55" s="25">
         <f>MAX(0, E55-F55)</f>
@@ -7722,10 +7722,10 @@
         <v/>
       </c>
       <c r="I55" s="25" t="n">
-        <v>126</v>
+        <v>177</v>
       </c>
       <c r="J55" s="25" t="n">
-        <v>104</v>
+        <v>154</v>
       </c>
       <c r="K55" s="25">
         <f>MAX(0, I55-J55)</f>
@@ -7750,10 +7750,10 @@
         <v/>
       </c>
       <c r="Q55" s="25" t="n">
-        <v>177</v>
+        <v>126</v>
       </c>
       <c r="R55" s="25" t="n">
-        <v>154</v>
+        <v>104</v>
       </c>
       <c r="S55" s="25">
         <f>MAX(0, Q55-R55)</f>
@@ -7764,10 +7764,10 @@
         <v/>
       </c>
       <c r="U55" s="25" t="n">
-        <v>175</v>
+        <v>123</v>
       </c>
       <c r="V55" s="25" t="n">
-        <v>149</v>
+        <v>113</v>
       </c>
       <c r="W55" s="25">
         <f>MAX(0, U55-V55)</f>
@@ -7814,10 +7814,10 @@
         </is>
       </c>
       <c r="E56" s="22" t="n">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="F56" s="22" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="G56" s="22">
         <f>MAX(0, E56-F56)</f>
@@ -7828,10 +7828,10 @@
         <v/>
       </c>
       <c r="I56" s="22" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="J56" s="22" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="K56" s="22">
         <f>MAX(0, I56-J56)</f>
@@ -7856,10 +7856,10 @@
         <v/>
       </c>
       <c r="Q56" s="22" t="n">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="R56" s="22" t="n">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="S56" s="22">
         <f>MAX(0, Q56-R56)</f>
@@ -7870,10 +7870,10 @@
         <v/>
       </c>
       <c r="U56" s="22" t="n">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="V56" s="22" t="n">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="W56" s="22">
         <f>MAX(0, U56-V56)</f>
@@ -7920,10 +7920,10 @@
         </is>
       </c>
       <c r="E57" s="25" t="n">
-        <v>106</v>
+        <v>173</v>
       </c>
       <c r="F57" s="25" t="n">
-        <v>91</v>
+        <v>149</v>
       </c>
       <c r="G57" s="25">
         <f>MAX(0, E57-F57)</f>
@@ -7934,10 +7934,10 @@
         <v/>
       </c>
       <c r="I57" s="25" t="n">
-        <v>112</v>
+        <v>164</v>
       </c>
       <c r="J57" s="25" t="n">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="K57" s="25">
         <f>MAX(0, I57-J57)</f>
@@ -7962,10 +7962,10 @@
         <v/>
       </c>
       <c r="Q57" s="25" t="n">
-        <v>164</v>
+        <v>112</v>
       </c>
       <c r="R57" s="25" t="n">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="S57" s="25">
         <f>MAX(0, Q57-R57)</f>
@@ -7976,10 +7976,10 @@
         <v/>
       </c>
       <c r="U57" s="25" t="n">
-        <v>173</v>
+        <v>106</v>
       </c>
       <c r="V57" s="25" t="n">
-        <v>149</v>
+        <v>91</v>
       </c>
       <c r="W57" s="25">
         <f>MAX(0, U57-V57)</f>
@@ -8026,10 +8026,10 @@
         </is>
       </c>
       <c r="E58" s="22" t="n">
-        <v>128</v>
+        <v>233</v>
       </c>
       <c r="F58" s="22" t="n">
-        <v>103</v>
+        <v>198</v>
       </c>
       <c r="G58" s="22">
         <f>MAX(0, E58-F58)</f>
@@ -8040,10 +8040,10 @@
         <v/>
       </c>
       <c r="I58" s="22" t="n">
-        <v>118</v>
+        <v>230</v>
       </c>
       <c r="J58" s="22" t="n">
-        <v>101</v>
+        <v>186</v>
       </c>
       <c r="K58" s="22">
         <f>MAX(0, I58-J58)</f>
@@ -8068,10 +8068,10 @@
         <v/>
       </c>
       <c r="Q58" s="22" t="n">
-        <v>230</v>
+        <v>118</v>
       </c>
       <c r="R58" s="22" t="n">
-        <v>186</v>
+        <v>101</v>
       </c>
       <c r="S58" s="22">
         <f>MAX(0, Q58-R58)</f>
@@ -8082,10 +8082,10 @@
         <v/>
       </c>
       <c r="U58" s="22" t="n">
-        <v>233</v>
+        <v>128</v>
       </c>
       <c r="V58" s="22" t="n">
-        <v>198</v>
+        <v>103</v>
       </c>
       <c r="W58" s="22">
         <f>MAX(0, U58-V58)</f>
@@ -8132,10 +8132,10 @@
         </is>
       </c>
       <c r="E59" s="25" t="n">
-        <v>106</v>
+        <v>172</v>
       </c>
       <c r="F59" s="25" t="n">
-        <v>94</v>
+        <v>145</v>
       </c>
       <c r="G59" s="25">
         <f>MAX(0, E59-F59)</f>
@@ -8146,10 +8146,10 @@
         <v/>
       </c>
       <c r="I59" s="25" t="n">
-        <v>118</v>
+        <v>168</v>
       </c>
       <c r="J59" s="25" t="n">
-        <v>101</v>
+        <v>145</v>
       </c>
       <c r="K59" s="25">
         <f>MAX(0, I59-J59)</f>
@@ -8174,10 +8174,10 @@
         <v/>
       </c>
       <c r="Q59" s="25" t="n">
-        <v>168</v>
+        <v>118</v>
       </c>
       <c r="R59" s="25" t="n">
-        <v>145</v>
+        <v>101</v>
       </c>
       <c r="S59" s="25">
         <f>MAX(0, Q59-R59)</f>
@@ -8188,10 +8188,10 @@
         <v/>
       </c>
       <c r="U59" s="25" t="n">
-        <v>172</v>
+        <v>106</v>
       </c>
       <c r="V59" s="25" t="n">
-        <v>145</v>
+        <v>94</v>
       </c>
       <c r="W59" s="25">
         <f>MAX(0, U59-V59)</f>
@@ -8238,10 +8238,10 @@
         </is>
       </c>
       <c r="E60" s="22" t="n">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="F60" s="22" t="n">
-        <v>105</v>
+        <v>217</v>
       </c>
       <c r="G60" s="22">
         <f>MAX(0, E60-F60)</f>
@@ -8252,10 +8252,10 @@
         <v/>
       </c>
       <c r="I60" s="22" t="n">
-        <v>148</v>
+        <v>256</v>
       </c>
       <c r="J60" s="22" t="n">
-        <v>108</v>
+        <v>204</v>
       </c>
       <c r="K60" s="22">
         <f>MAX(0, I60-J60)</f>
@@ -8280,10 +8280,10 @@
         <v/>
       </c>
       <c r="Q60" s="22" t="n">
-        <v>256</v>
+        <v>148</v>
       </c>
       <c r="R60" s="22" t="n">
-        <v>204</v>
+        <v>108</v>
       </c>
       <c r="S60" s="22">
         <f>MAX(0, Q60-R60)</f>
@@ -8294,10 +8294,10 @@
         <v/>
       </c>
       <c r="U60" s="22" t="n">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="V60" s="22" t="n">
-        <v>217</v>
+        <v>105</v>
       </c>
       <c r="W60" s="22">
         <f>MAX(0, U60-V60)</f>
@@ -8344,7 +8344,7 @@
         </is>
       </c>
       <c r="E61" s="25" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F61" s="25" t="n">
         <v>76</v>
@@ -8358,10 +8358,10 @@
         <v/>
       </c>
       <c r="I61" s="25" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="J61" s="25" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="K61" s="25">
         <f>MAX(0, I61-J61)</f>
@@ -8386,10 +8386,10 @@
         <v/>
       </c>
       <c r="Q61" s="25" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="R61" s="25" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="S61" s="25">
         <f>MAX(0, Q61-R61)</f>
@@ -8400,7 +8400,7 @@
         <v/>
       </c>
       <c r="U61" s="25" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="V61" s="25" t="n">
         <v>76</v>
@@ -8450,10 +8450,10 @@
         </is>
       </c>
       <c r="E62" s="22" t="n">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="F62" s="22" t="n">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="G62" s="22">
         <f>MAX(0, E62-F62)</f>
@@ -8464,10 +8464,10 @@
         <v/>
       </c>
       <c r="I62" s="22" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="J62" s="22" t="n">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="K62" s="22">
         <f>MAX(0, I62-J62)</f>
@@ -8492,10 +8492,10 @@
         <v/>
       </c>
       <c r="Q62" s="22" t="n">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="R62" s="22" t="n">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="S62" s="22">
         <f>MAX(0, Q62-R62)</f>
@@ -8506,10 +8506,10 @@
         <v/>
       </c>
       <c r="U62" s="22" t="n">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="V62" s="22" t="n">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="W62" s="22">
         <f>MAX(0, U62-V62)</f>
@@ -8556,10 +8556,10 @@
         </is>
       </c>
       <c r="E63" s="25" t="n">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="F63" s="25" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="G63" s="25">
         <f>MAX(0, E63-F63)</f>
@@ -8570,10 +8570,10 @@
         <v/>
       </c>
       <c r="I63" s="25" t="n">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="J63" s="25" t="n">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="K63" s="25">
         <f>MAX(0, I63-J63)</f>
@@ -8598,10 +8598,10 @@
         <v/>
       </c>
       <c r="Q63" s="25" t="n">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="R63" s="25" t="n">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="S63" s="25">
         <f>MAX(0, Q63-R63)</f>
@@ -8612,10 +8612,10 @@
         <v/>
       </c>
       <c r="U63" s="25" t="n">
+        <v>135</v>
+      </c>
+      <c r="V63" s="25" t="n">
         <v>108</v>
-      </c>
-      <c r="V63" s="25" t="n">
-        <v>92</v>
       </c>
       <c r="W63" s="25">
         <f>MAX(0, U63-V63)</f>
@@ -8662,10 +8662,10 @@
         </is>
       </c>
       <c r="E64" s="22" t="n">
-        <v>152</v>
+        <v>206</v>
       </c>
       <c r="F64" s="22" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="G64" s="22">
         <f>MAX(0, E64-F64)</f>
@@ -8676,10 +8676,10 @@
         <v/>
       </c>
       <c r="I64" s="22" t="n">
-        <v>157</v>
+        <v>209</v>
       </c>
       <c r="J64" s="22" t="n">
-        <v>136</v>
+        <v>181</v>
       </c>
       <c r="K64" s="22">
         <f>MAX(0, I64-J64)</f>
@@ -8704,10 +8704,10 @@
         <v/>
       </c>
       <c r="Q64" s="22" t="n">
-        <v>209</v>
+        <v>157</v>
       </c>
       <c r="R64" s="22" t="n">
-        <v>181</v>
+        <v>136</v>
       </c>
       <c r="S64" s="22">
         <f>MAX(0, Q64-R64)</f>
@@ -8718,10 +8718,10 @@
         <v/>
       </c>
       <c r="U64" s="22" t="n">
-        <v>206</v>
+        <v>152</v>
       </c>
       <c r="V64" s="22" t="n">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="W64" s="22">
         <f>MAX(0, U64-V64)</f>
@@ -8768,10 +8768,10 @@
         </is>
       </c>
       <c r="E65" s="25" t="n">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="F65" s="25" t="n">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="G65" s="25">
         <f>MAX(0, E65-F65)</f>
@@ -8782,10 +8782,10 @@
         <v/>
       </c>
       <c r="I65" s="25" t="n">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="J65" s="25" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="K65" s="25">
         <f>MAX(0, I65-J65)</f>
@@ -8810,10 +8810,10 @@
         <v/>
       </c>
       <c r="Q65" s="25" t="n">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="R65" s="25" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="S65" s="25">
         <f>MAX(0, Q65-R65)</f>
@@ -8824,10 +8824,10 @@
         <v/>
       </c>
       <c r="U65" s="25" t="n">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="V65" s="25" t="n">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="W65" s="25">
         <f>MAX(0, U65-V65)</f>
@@ -8874,10 +8874,10 @@
         </is>
       </c>
       <c r="E66" s="22" t="n">
-        <v>150</v>
+        <v>212</v>
       </c>
       <c r="F66" s="22" t="n">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="G66" s="22">
         <f>MAX(0, E66-F66)</f>
@@ -8888,10 +8888,10 @@
         <v/>
       </c>
       <c r="I66" s="22" t="n">
-        <v>161</v>
+        <v>212</v>
       </c>
       <c r="J66" s="22" t="n">
-        <v>136</v>
+        <v>174</v>
       </c>
       <c r="K66" s="22">
         <f>MAX(0, I66-J66)</f>
@@ -8916,10 +8916,10 @@
         <v/>
       </c>
       <c r="Q66" s="22" t="n">
-        <v>212</v>
+        <v>161</v>
       </c>
       <c r="R66" s="22" t="n">
-        <v>174</v>
+        <v>136</v>
       </c>
       <c r="S66" s="22">
         <f>MAX(0, Q66-R66)</f>
@@ -8930,10 +8930,10 @@
         <v/>
       </c>
       <c r="U66" s="22" t="n">
-        <v>212</v>
+        <v>150</v>
       </c>
       <c r="V66" s="22" t="n">
-        <v>181</v>
+        <v>132</v>
       </c>
       <c r="W66" s="22">
         <f>MAX(0, U66-V66)</f>
@@ -8980,10 +8980,10 @@
         </is>
       </c>
       <c r="E67" s="25" t="n">
-        <v>197</v>
+        <v>138</v>
       </c>
       <c r="F67" s="25" t="n">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="G67" s="25">
         <f>MAX(0, E67-F67)</f>
@@ -8994,10 +8994,10 @@
         <v/>
       </c>
       <c r="I67" s="25" t="n">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="J67" s="25" t="n">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="K67" s="25">
         <f>MAX(0, I67-J67)</f>
@@ -9022,10 +9022,10 @@
         <v/>
       </c>
       <c r="Q67" s="25" t="n">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="R67" s="25" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="S67" s="25">
         <f>MAX(0, Q67-R67)</f>
@@ -9036,10 +9036,10 @@
         <v/>
       </c>
       <c r="U67" s="25" t="n">
-        <v>138</v>
+        <v>197</v>
       </c>
       <c r="V67" s="25" t="n">
-        <v>122</v>
+        <v>165</v>
       </c>
       <c r="W67" s="25">
         <f>MAX(0, U67-V67)</f>
@@ -9086,10 +9086,10 @@
         </is>
       </c>
       <c r="E68" s="22" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F68" s="22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G68" s="22">
         <f>MAX(0, E68-F68)</f>
@@ -9100,10 +9100,10 @@
         <v/>
       </c>
       <c r="I68" s="22" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="J68" s="22" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="K68" s="22">
         <f>MAX(0, I68-J68)</f>
@@ -9128,10 +9128,10 @@
         <v/>
       </c>
       <c r="Q68" s="22" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="R68" s="22" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="S68" s="22">
         <f>MAX(0, Q68-R68)</f>
@@ -9142,10 +9142,10 @@
         <v/>
       </c>
       <c r="U68" s="22" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="V68" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W68" s="22">
         <f>MAX(0, U68-V68)</f>
@@ -9192,10 +9192,10 @@
         </is>
       </c>
       <c r="E69" s="25" t="n">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="F69" s="25" t="n">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="G69" s="25">
         <f>MAX(0, E69-F69)</f>
@@ -9206,10 +9206,10 @@
         <v/>
       </c>
       <c r="I69" s="25" t="n">
-        <v>32</v>
+        <v>89</v>
       </c>
       <c r="J69" s="25" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="K69" s="25">
         <f>MAX(0, I69-J69)</f>
@@ -9234,10 +9234,10 @@
         <v/>
       </c>
       <c r="Q69" s="25" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="R69" s="25" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="S69" s="25">
         <f>MAX(0, Q69-R69)</f>
@@ -9248,10 +9248,10 @@
         <v/>
       </c>
       <c r="U69" s="25" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="V69" s="25" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="W69" s="25">
         <f>MAX(0, U69-V69)</f>
@@ -9298,10 +9298,10 @@
         </is>
       </c>
       <c r="E70" s="22" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F70" s="22" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G70" s="22">
         <f>MAX(0, E70-F70)</f>
@@ -9312,10 +9312,10 @@
         <v/>
       </c>
       <c r="I70" s="22" t="n">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="J70" s="22" t="n">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="K70" s="22">
         <f>MAX(0, I70-J70)</f>
@@ -9340,10 +9340,10 @@
         <v/>
       </c>
       <c r="Q70" s="22" t="n">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="R70" s="22" t="n">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="S70" s="22">
         <f>MAX(0, Q70-R70)</f>
@@ -9354,10 +9354,10 @@
         <v/>
       </c>
       <c r="U70" s="22" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V70" s="22" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W70" s="22">
         <f>MAX(0, U70-V70)</f>
@@ -9404,10 +9404,10 @@
         </is>
       </c>
       <c r="E71" s="25" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F71" s="25" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="G71" s="25">
         <f>MAX(0, E71-F71)</f>
@@ -9418,10 +9418,10 @@
         <v/>
       </c>
       <c r="I71" s="25" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="J71" s="25" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="K71" s="25">
         <f>MAX(0, I71-J71)</f>
@@ -9446,10 +9446,10 @@
         <v/>
       </c>
       <c r="Q71" s="25" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="R71" s="25" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="S71" s="25">
         <f>MAX(0, Q71-R71)</f>
@@ -9460,10 +9460,10 @@
         <v/>
       </c>
       <c r="U71" s="25" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="V71" s="25" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W71" s="25">
         <f>MAX(0, U71-V71)</f>
@@ -9510,10 +9510,10 @@
         </is>
       </c>
       <c r="E72" s="22" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F72" s="22" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G72" s="22">
         <f>MAX(0, E72-F72)</f>
@@ -9524,10 +9524,10 @@
         <v/>
       </c>
       <c r="I72" s="22" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J72" s="22" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K72" s="22">
         <f>MAX(0, I72-J72)</f>
@@ -9552,10 +9552,10 @@
         <v/>
       </c>
       <c r="Q72" s="22" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="R72" s="22" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="S72" s="22">
         <f>MAX(0, Q72-R72)</f>
@@ -9566,10 +9566,10 @@
         <v/>
       </c>
       <c r="U72" s="22" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="V72" s="22" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="W72" s="22">
         <f>MAX(0, U72-V72)</f>
@@ -9616,10 +9616,10 @@
         </is>
       </c>
       <c r="E73" s="25" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="F73" s="25" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="G73" s="25">
         <f>MAX(0, E73-F73)</f>
@@ -9630,10 +9630,10 @@
         <v/>
       </c>
       <c r="I73" s="25" t="n">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="J73" s="25" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="K73" s="25">
         <f>MAX(0, I73-J73)</f>
@@ -9658,10 +9658,10 @@
         <v/>
       </c>
       <c r="Q73" s="25" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="R73" s="25" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="S73" s="25">
         <f>MAX(0, Q73-R73)</f>
@@ -9672,10 +9672,10 @@
         <v/>
       </c>
       <c r="U73" s="25" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="V73" s="25" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="W73" s="25">
         <f>MAX(0, U73-V73)</f>
@@ -9722,10 +9722,10 @@
         </is>
       </c>
       <c r="E74" s="22" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F74" s="22" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="G74" s="22">
         <f>MAX(0, E74-F74)</f>
@@ -9736,10 +9736,10 @@
         <v/>
       </c>
       <c r="I74" s="22" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="J74" s="22" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="K74" s="22">
         <f>MAX(0, I74-J74)</f>
@@ -9764,10 +9764,10 @@
         <v/>
       </c>
       <c r="Q74" s="22" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="R74" s="22" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="S74" s="22">
         <f>MAX(0, Q74-R74)</f>
@@ -9778,10 +9778,10 @@
         <v/>
       </c>
       <c r="U74" s="22" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="V74" s="22" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="W74" s="22">
         <f>MAX(0, U74-V74)</f>
@@ -9828,10 +9828,10 @@
         </is>
       </c>
       <c r="E75" s="25" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="F75" s="25" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G75" s="25">
         <f>MAX(0, E75-F75)</f>
@@ -9842,10 +9842,10 @@
         <v/>
       </c>
       <c r="I75" s="25" t="n">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="J75" s="25" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="K75" s="25">
         <f>MAX(0, I75-J75)</f>
@@ -9870,10 +9870,10 @@
         <v/>
       </c>
       <c r="Q75" s="25" t="n">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="R75" s="25" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="S75" s="25">
         <f>MAX(0, Q75-R75)</f>
@@ -9884,10 +9884,10 @@
         <v/>
       </c>
       <c r="U75" s="25" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="V75" s="25" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="W75" s="25">
         <f>MAX(0, U75-V75)</f>
@@ -9934,10 +9934,10 @@
         </is>
       </c>
       <c r="E76" s="22" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F76" s="22" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G76" s="22">
         <f>MAX(0, E76-F76)</f>
@@ -9948,10 +9948,10 @@
         <v/>
       </c>
       <c r="I76" s="22" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J76" s="22" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="K76" s="22">
         <f>MAX(0, I76-J76)</f>
@@ -9976,10 +9976,10 @@
         <v/>
       </c>
       <c r="Q76" s="22" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="R76" s="22" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="S76" s="22">
         <f>MAX(0, Q76-R76)</f>
@@ -9990,10 +9990,10 @@
         <v/>
       </c>
       <c r="U76" s="22" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="V76" s="22" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="W76" s="22">
         <f>MAX(0, U76-V76)</f>
@@ -10040,10 +10040,10 @@
         </is>
       </c>
       <c r="E77" s="25" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F77" s="25" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G77" s="25">
         <f>MAX(0, E77-F77)</f>
@@ -10054,10 +10054,10 @@
         <v/>
       </c>
       <c r="I77" s="25" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="J77" s="25" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="K77" s="25">
         <f>MAX(0, I77-J77)</f>
@@ -10082,10 +10082,10 @@
         <v/>
       </c>
       <c r="Q77" s="25" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="R77" s="25" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="S77" s="25">
         <f>MAX(0, Q77-R77)</f>
@@ -10096,10 +10096,10 @@
         <v/>
       </c>
       <c r="U77" s="25" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="V77" s="25" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="W77" s="25">
         <f>MAX(0, U77-V77)</f>
@@ -10146,10 +10146,10 @@
         </is>
       </c>
       <c r="E78" s="22" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F78" s="22" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="G78" s="22">
         <f>MAX(0, E78-F78)</f>
@@ -10160,10 +10160,10 @@
         <v/>
       </c>
       <c r="I78" s="22" t="n">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="J78" s="22" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="K78" s="22">
         <f>MAX(0, I78-J78)</f>
@@ -10188,10 +10188,10 @@
         <v/>
       </c>
       <c r="Q78" s="22" t="n">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="R78" s="22" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="S78" s="22">
         <f>MAX(0, Q78-R78)</f>
@@ -10202,10 +10202,10 @@
         <v/>
       </c>
       <c r="U78" s="22" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="V78" s="22" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="W78" s="22">
         <f>MAX(0, U78-V78)</f>
@@ -10252,10 +10252,10 @@
         </is>
       </c>
       <c r="E79" s="25" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F79" s="25" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G79" s="25">
         <f>MAX(0, E79-F79)</f>
@@ -10266,10 +10266,10 @@
         <v/>
       </c>
       <c r="I79" s="25" t="n">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="J79" s="25" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="K79" s="25">
         <f>MAX(0, I79-J79)</f>
@@ -10294,10 +10294,10 @@
         <v/>
       </c>
       <c r="Q79" s="25" t="n">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="R79" s="25" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="S79" s="25">
         <f>MAX(0, Q79-R79)</f>
@@ -10308,10 +10308,10 @@
         <v/>
       </c>
       <c r="U79" s="25" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="V79" s="25" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="W79" s="25">
         <f>MAX(0, U79-V79)</f>
@@ -10358,10 +10358,10 @@
         </is>
       </c>
       <c r="E80" s="22" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F80" s="22" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="G80" s="22">
         <f>MAX(0, E80-F80)</f>
@@ -10372,10 +10372,10 @@
         <v/>
       </c>
       <c r="I80" s="22" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="J80" s="22" t="n">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="K80" s="22">
         <f>MAX(0, I80-J80)</f>
@@ -10400,10 +10400,10 @@
         <v/>
       </c>
       <c r="Q80" s="22" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="R80" s="22" t="n">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="S80" s="22">
         <f>MAX(0, Q80-R80)</f>
@@ -10414,10 +10414,10 @@
         <v/>
       </c>
       <c r="U80" s="22" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="V80" s="22" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="W80" s="22">
         <f>MAX(0, U80-V80)</f>
@@ -10464,10 +10464,10 @@
         </is>
       </c>
       <c r="E81" s="25" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F81" s="25" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G81" s="25">
         <f>MAX(0, E81-F81)</f>
@@ -10478,10 +10478,10 @@
         <v/>
       </c>
       <c r="I81" s="25" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="J81" s="25" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="K81" s="25">
         <f>MAX(0, I81-J81)</f>
@@ -10506,10 +10506,10 @@
         <v/>
       </c>
       <c r="Q81" s="25" t="n">
+        <v>55</v>
+      </c>
+      <c r="R81" s="25" t="n">
         <v>36</v>
-      </c>
-      <c r="R81" s="25" t="n">
-        <v>32</v>
       </c>
       <c r="S81" s="25">
         <f>MAX(0, Q81-R81)</f>
@@ -10520,10 +10520,10 @@
         <v/>
       </c>
       <c r="U81" s="25" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="V81" s="25" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="W81" s="25">
         <f>MAX(0, U81-V81)</f>
@@ -10570,10 +10570,10 @@
         </is>
       </c>
       <c r="E82" s="22" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F82" s="22" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G82" s="22">
         <f>MAX(0, E82-F82)</f>
@@ -10584,10 +10584,10 @@
         <v/>
       </c>
       <c r="I82" s="22" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J82" s="22" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="K82" s="22">
         <f>MAX(0, I82-J82)</f>
@@ -10612,10 +10612,10 @@
         <v/>
       </c>
       <c r="Q82" s="22" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="R82" s="22" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="S82" s="22">
         <f>MAX(0, Q82-R82)</f>
@@ -10626,10 +10626,10 @@
         <v/>
       </c>
       <c r="U82" s="22" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="V82" s="22" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W82" s="22">
         <f>MAX(0, U82-V82)</f>
@@ -10676,10 +10676,10 @@
         </is>
       </c>
       <c r="E83" s="25" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="F83" s="25" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G83" s="25">
         <f>MAX(0, E83-F83)</f>
@@ -10690,10 +10690,10 @@
         <v/>
       </c>
       <c r="I83" s="25" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J83" s="25" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="K83" s="25">
         <f>MAX(0, I83-J83)</f>
@@ -10718,10 +10718,10 @@
         <v/>
       </c>
       <c r="Q83" s="25" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="R83" s="25" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="S83" s="25">
         <f>MAX(0, Q83-R83)</f>
@@ -10732,10 +10732,10 @@
         <v/>
       </c>
       <c r="U83" s="25" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="V83" s="25" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="W83" s="25">
         <f>MAX(0, U83-V83)</f>
@@ -10782,10 +10782,10 @@
         </is>
       </c>
       <c r="E84" s="22" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F84" s="22" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="G84" s="22">
         <f>MAX(0, E84-F84)</f>
@@ -10796,10 +10796,10 @@
         <v/>
       </c>
       <c r="I84" s="22" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J84" s="22" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="K84" s="22">
         <f>MAX(0, I84-J84)</f>
@@ -10824,10 +10824,10 @@
         <v/>
       </c>
       <c r="Q84" s="22" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R84" s="22" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="S84" s="22">
         <f>MAX(0, Q84-R84)</f>
@@ -10838,10 +10838,10 @@
         <v/>
       </c>
       <c r="U84" s="22" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="V84" s="22" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="W84" s="22">
         <f>MAX(0, U84-V84)</f>
@@ -10888,10 +10888,10 @@
         </is>
       </c>
       <c r="E85" s="25" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F85" s="25" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G85" s="25">
         <f>MAX(0, E85-F85)</f>
@@ -10902,10 +10902,10 @@
         <v/>
       </c>
       <c r="I85" s="25" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="J85" s="25" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="K85" s="25">
         <f>MAX(0, I85-J85)</f>
@@ -10930,10 +10930,10 @@
         <v/>
       </c>
       <c r="Q85" s="25" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="R85" s="25" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="S85" s="25">
         <f>MAX(0, Q85-R85)</f>
@@ -10944,10 +10944,10 @@
         <v/>
       </c>
       <c r="U85" s="25" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="V85" s="25" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="W85" s="25">
         <f>MAX(0, U85-V85)</f>
@@ -10994,10 +10994,10 @@
         </is>
       </c>
       <c r="E86" s="22" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="F86" s="22" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="G86" s="22">
         <f>MAX(0, E86-F86)</f>
@@ -11050,10 +11050,10 @@
         <v/>
       </c>
       <c r="U86" s="22" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="V86" s="22" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="W86" s="22">
         <f>MAX(0, U86-V86)</f>

</xml_diff>